<commit_message>
Daily EOD data and reports for 2026-09-29
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260929.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260929.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.85</v>
+        <v>1.84</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.015</v>
+        <v>-0.025</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-1.34%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>283384.85</v>
+        <v>281853.04</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-2297.71</v>
+        <v>-3829.52</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.57</v>
+        <v>2.58</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.02</v>
+        <v>-0.01</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.39%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>179900</v>
+        <v>180600</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-1400</v>
+        <v>-700</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>60.31</v>
+        <v>60.33</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.51</v>
+        <v>0.53</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.85%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>482480</v>
+        <v>482640</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>4080</v>
+        <v>4240</v>
       </c>
     </row>
     <row r="7">
@@ -596,10 +596,10 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>150.5</v>
+        <v>150.51</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-1.02</v>
+        <v>-1.01</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0</v>
+        <v>0.895</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.89</v>
+        <v>0.005</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.56%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0</v>
+        <v>8950</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-8900</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>182.1</v>
+        <v>182.51</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.19</v>
+        <v>0.6</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>728400</v>
+        <v>730040</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>760</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="11">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>15.47</v>
+        <v>15.5</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.55</v>
+        <v>-0.52</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>-3.25%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>47106.15</v>
+        <v>47197.5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-1674.75</v>
+        <v>-1583.4</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.094</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.093</v>
+        <v>0.001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>884.73</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-875.3200000000001</v>
+        <v>9.41</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.89</v>
+        <v>34.87</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.43%</t>
+          <t>-0.49%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.36</v>
+        <v>31.29</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.41</v>
+        <v>-0.48</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-1.29%</t>
+          <t>-1.51%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40391.68</v>
+        <v>40301.52</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-528.08</v>
+        <v>-618.24</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1766162.68</v>
+        <v>1776966.79</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-13096.31</v>
+        <v>-2292.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>